<commit_message>
Amend WBD ($29→$30) and ACN ($215→$170) limits
WBD: confirmed Paramount takeout $31; new limit sits below
takeout to capture arb if deal-risk spread narrows.
ACN: post-Q3 print (revenue miss, bookings down YoY, FY26
guide cut to 3-4%), $215 was inert; new $170 targets recovery
to no-news pricing. Logged in open_orders.md, journal.md,
company_notes.csv (+xlsx regenerated).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R9hEPtpSbfMJBEZfn8QAcQ
</commit_message>
<xml_diff>
--- a/portfolio/company_notes.xlsx
+++ b/portfolio/company_notes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Company Notes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Company Notes'!$A$1:$H$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Company Notes'!$A$1:$H$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1117,8 +1117,84 @@
       </c>
       <c r="H17" s="3" t="n"/>
     </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>WBD</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>limit amended $29 → $30</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed Paramount takeout $31 + ticking; spot $27; $30 sits below takeout, captures arb if deal-risk spread narrows (10% give-up at $30 vs 3.3% at $31)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Patient exit. Wants more of the arb than $29 would have captured. If spread doesn't narrow, hold to deal close.</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Monitor regulatory milestones; if spread holds wide for 90 days, accept holding to close.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>WBD IR</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n"/>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>ACN</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>limit amended $215 → $170</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Post Q3 FY26 miss + guide cut to 3-4%; spot $156; intraday high $166.87; $170 = +9% above spot, ~$3 above today's high</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Patient exit targeting recovery to no-news pricing. Locks ~13% loss if filled.</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Watch 60-90 days. If drifts $145-160 and no fill, re-evaluate.</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>ChartMill / Investing.com</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H17"/>
+  <autoFilter ref="A1:H19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Amend SRL limit (185 @ A$10 → 150 @ A$12.50)
Old order sat -41% below market — crash-only trigger. New order
sits -26% below as a moderate-pullback add level, with size
trimmed to keep dollar exposure roughly the same. Adding to a
+90% speculative position; the parallel "take some off" trim
decision on the existing 60sh remains open.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R9hEPtpSbfMJBEZfn8QAcQ
</commit_message>
<xml_diff>
--- a/portfolio/company_notes.xlsx
+++ b/portfolio/company_notes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Company Notes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Company Notes'!$A$1:$H$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Company Notes'!$A$1:$H$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1193,8 +1193,46 @@
       </c>
       <c r="H19" s="3" t="n"/>
     </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>SRL</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>limit amended 185@A$10 → 150@A$12.50</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Spot A$16.87; old limit -41% below (crash-only), new -26% below (moderate pullback); size cut so dollar add stays similar; if filled blended avg ~A$11.47 across 210sh</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Keeps add-to-winner on the table at more realistic level. Adds more size to a +90% speculative position.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Trim trigger on existing 60sh still unresolved — write a separate journal rule (e.g., trim 30sh if &gt; A$20).</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H19"/>
+  <autoFilter ref="A1:H20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Log SRL thesis (scandium pure-play) + RIO/REMX context
User confirmed sticking with SRL as concentrated scandium
exposure — explicit exception to no-unprofitable-companies
rule, justified as commodity vehicle. Adds context rows for
RIO (incidental Sc beta via Sorel-Tracy byproduct) and REMX
(diversified critical-minerals alternative, passed).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R9hEPtpSbfMJBEZfn8QAcQ
</commit_message>
<xml_diff>
--- a/portfolio/company_notes.xlsx
+++ b/portfolio/company_notes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Company Notes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Company Notes'!$A$1:$H$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Company Notes'!$A$1:$H$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1231,8 +1231,122 @@
       </c>
       <c r="H20" s="2" t="n"/>
     </row>
+    <row r="21" ht="90" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>SRL</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>thesis confirmed — scandium pure-play</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Cost A$8.89, spot A$16.87 (+89.9%); pre-revenue developer, FID H2 2026; Lockheed Martin Syerston offtake option (25% of annual output / 5 years); global scandium supply only 15-40 t/yr; only profitable Sc-exposed name is RIO via Sorel-Tracy byproduct (tiny share of $50B+ topline = near-zero Sc beta); REMX = diversified critical-minerals alternative but dilutes Sc-specific bet</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>User sticking with SRL as the concentrated scandium pure-play. Explicit exception to "no unprofitable companies" rule, justified as commodity vehicle (not fundamental equity). Conviction is scandium-specific (Lockheed Martin offtake, Western supply security) NOT broader critical minerals (which would point to REMX).</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>1) Add profitability gate + commodity-vehicle exception to strategy.md. 2) Define trim/add rules for SRL (currently open BUY 150 @ A$12.50). 3) Trim trigger on existing +90% position still unwritten.</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>USGS / INN / Stocks Down Under</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="n"/>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>RIO</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>incidental scandium exposure</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Position 20 sh @ £64.98 cost / ~£77 spot; £1,541 / ~$2,069 USD; RIO commercially produces scandium oxide at Sorel-Tracy Québec since mid-2021 as TiO2 byproduct</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>User did not realize RIO gives any scandium exposure. Beta to Sc price is near-zero (rounding error on $50B+ topline). Notable as context — user is already long Sc beta from two angles (RIO incidental + SRL concentrated).</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>No action — informational note that connects RIO to the scandium thesis.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>INN scandium primer</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="n"/>
+    </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>REMX</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>alternative considered, passed</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>VanEck Rare Earth/Strategic Metals ETF; basket includes Lynas, Iluka, Almonty, Lithium Americas, AMG Critical Materials; Australia 24%, Canada 9.5%; mixed profitability</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Considered as the "diversified critical-minerals" expression. User passed — thesis is scandium-specific, not broader critical-minerals, so REMX dilutes the bet.</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Watchlist note: REMX is the right vehicle if thesis ever broadens from scandium-specific to critical-minerals-as-category.</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>VanEck NPORT filing</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H20"/>
+  <autoFilter ref="A1:H23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>